<commit_message>
Add iteration #31: market rent from in-place when source lacks a market column
New RollConfig.market_from_inplace toggle (default False): when a source
has no market/asking-rent column, set every unit's market rent to the max
in-place rent of the same unit type ('achievable market' proxy), instead
of echoing each unit's own in-place. Supersedes the vacant-only derivation
when on. derive.py _apply_market_from_inplace, gated in apply_deal_rules.
Enabled on Nova and Greenville (both lack a market column); deals with real
market rents are untouched. Nova Unit-Mix market total now 164,440 vs
in-place 113,985. Heritage regression unchanged (ALL VALUES MATCH).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QgY3cyE49yD2oQoBHHNQL4
</commit_message>
<xml_diff>
--- a/examples/outputs/Birgo RR Exhibits - Greenville Portfoliov07.28.26.xlsx
+++ b/examples/outputs/Birgo RR Exhibits - Greenville Portfoliov07.28.26.xlsx
@@ -906,10 +906,10 @@
         <v>0</v>
       </c>
       <c r="J6" s="11" t="n">
-        <v>22629.83</v>
+        <v>29268.39999999999</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>1131.4915</v>
+        <v>1463.419999999999</v>
       </c>
       <c r="L6" s="12" t="n">
         <v>0</v>
@@ -955,10 +955,10 @@
         <v>0</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>28277.85</v>
+        <v>34960</v>
       </c>
       <c r="K7" s="11" t="n">
-        <v>1229.471739130435</v>
+        <v>1520</v>
       </c>
       <c r="L7" s="12" t="n">
         <v>0</v>
@@ -1004,10 +1004,10 @@
         <v>0</v>
       </c>
       <c r="J8" s="11" t="n">
-        <v>17453.9</v>
+        <v>22188</v>
       </c>
       <c r="K8" s="11" t="n">
-        <v>1454.491666666667</v>
+        <v>1849</v>
       </c>
       <c r="L8" s="12" t="n">
         <v>0</v>
@@ -1053,10 +1053,10 @@
         <v>0</v>
       </c>
       <c r="J9" s="11" t="n">
-        <v>20941.22</v>
+        <v>24102</v>
       </c>
       <c r="K9" s="11" t="n">
-        <v>1163.401111111111</v>
+        <v>1339</v>
       </c>
       <c r="L9" s="12" t="n">
         <v>0</v>
@@ -1099,10 +1099,10 @@
         <v>0</v>
       </c>
       <c r="J10" s="17" t="n">
-        <v>89302.80000000002</v>
+        <v>110518.4</v>
       </c>
       <c r="K10" s="17" t="n">
-        <v>1223.326027397261</v>
+        <v>1513.950684931506</v>
       </c>
       <c r="L10" s="18" t="n">
         <v>0</v>
@@ -1212,7 +1212,7 @@
       <c r="E19" s="20" t="n"/>
       <c r="F19" s="20" t="n"/>
       <c r="G19" s="24" t="n">
-        <v>1071633.6</v>
+        <v>1326220.8</v>
       </c>
     </row>
     <row r="20">
@@ -1315,7 +1315,7 @@
         </is>
       </c>
       <c r="W48" s="27" t="n">
-        <v>89302.80000000002</v>
+        <v>110518.4</v>
       </c>
     </row>
     <row r="49">
@@ -1590,16 +1590,16 @@
         <v>0</v>
       </c>
       <c r="J7" s="11" t="n">
-        <v>1131.4915</v>
+        <v>1463.419999999999</v>
       </c>
       <c r="K7" s="38" t="n">
-        <v>1117.35947368421</v>
+        <v>1463.419999999999</v>
       </c>
       <c r="L7" s="11" t="n">
         <v>1117.35947368421</v>
       </c>
       <c r="M7" s="39" t="n">
-        <v>1</v>
+        <v>0.7635261740882391</v>
       </c>
       <c r="N7" s="38" t="inlineStr">
         <is>
@@ -1666,16 +1666,16 @@
         <v>0</v>
       </c>
       <c r="J8" s="11" t="n">
-        <v>1229.471739130435</v>
+        <v>1520</v>
       </c>
       <c r="K8" s="38" t="n">
-        <v>1228.538636363636</v>
+        <v>1520</v>
       </c>
       <c r="L8" s="11" t="n">
         <v>1228.538636363636</v>
       </c>
       <c r="M8" s="39" t="n">
-        <v>1</v>
+        <v>0.8082491028708133</v>
       </c>
       <c r="N8" s="38" t="n">
         <v>1250</v>
@@ -1736,16 +1736,16 @@
         <v>0</v>
       </c>
       <c r="J9" s="11" t="n">
-        <v>1454.491666666667</v>
+        <v>1849</v>
       </c>
       <c r="K9" s="38" t="n">
-        <v>1454.491666666667</v>
+        <v>1849</v>
       </c>
       <c r="L9" s="11" t="n">
         <v>1454.491666666667</v>
       </c>
       <c r="M9" s="39" t="n">
-        <v>1</v>
+        <v>0.7866369208581215</v>
       </c>
       <c r="N9" s="38" t="n">
         <v>1600</v>
@@ -1802,16 +1802,16 @@
         <v>0</v>
       </c>
       <c r="J10" s="11" t="n">
-        <v>1163.401111111111</v>
+        <v>1339</v>
       </c>
       <c r="K10" s="38" t="n">
-        <v>1152.57625</v>
+        <v>1339</v>
       </c>
       <c r="L10" s="11" t="n">
         <v>1152.57625</v>
       </c>
       <c r="M10" s="39" t="n">
-        <v>1</v>
+        <v>0.8607738984316653</v>
       </c>
       <c r="N10" s="38" t="n">
         <v>1225</v>
@@ -1865,16 +1865,16 @@
         <v>0</v>
       </c>
       <c r="J11" s="17" t="n">
-        <v>1223.326027397261</v>
+        <v>1513.950684931506</v>
       </c>
       <c r="K11" s="42" t="n">
-        <v>1219.605797101449</v>
+        <v>1519.666376811594</v>
       </c>
       <c r="L11" s="17" t="n">
         <v>1219.605797101449</v>
       </c>
       <c r="M11" s="43" t="n">
-        <v>1</v>
+        <v>0.8025483854293728</v>
       </c>
       <c r="N11" s="42" t="inlineStr">
         <is>
@@ -1991,7 +1991,7 @@
         </is>
       </c>
       <c r="AB65" s="27" t="n">
-        <v>89302.80000000002</v>
+        <v>110518.4</v>
       </c>
     </row>
     <row r="66">
@@ -2169,10 +2169,10 @@
         <v>0</v>
       </c>
       <c r="J6" s="11" t="n">
-        <v>89302.80000000002</v>
+        <v>110518.4</v>
       </c>
       <c r="K6" s="11" t="n">
-        <v>1223.326027397261</v>
+        <v>1513.950684931506</v>
       </c>
       <c r="L6" s="12" t="n">
         <v>0</v>
@@ -2215,10 +2215,10 @@
         <v>0</v>
       </c>
       <c r="J7" s="17" t="n">
-        <v>89302.80000000002</v>
+        <v>110518.4</v>
       </c>
       <c r="K7" s="17" t="n">
-        <v>1223.326027397261</v>
+        <v>1513.950684931506</v>
       </c>
       <c r="L7" s="18" t="n">
         <v>0</v>
@@ -2330,7 +2330,7 @@
       <c r="E16" s="20" t="n"/>
       <c r="F16" s="20" t="n"/>
       <c r="G16" s="24" t="n">
-        <v>1071633.6</v>
+        <v>1326220.8</v>
       </c>
     </row>
     <row r="17">
@@ -2785,7 +2785,7 @@
         </is>
       </c>
       <c r="U8" s="58" t="n">
-        <v>1250</v>
+        <v>1339</v>
       </c>
       <c r="V8" s="58" t="n">
         <v>0</v>
@@ -2837,7 +2837,7 @@
         </is>
       </c>
       <c r="U9" s="58" t="n">
-        <v>1250</v>
+        <v>1339</v>
       </c>
       <c r="V9" s="58" t="n">
         <v>0</v>
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="U10" s="58" t="n">
-        <v>1250</v>
+        <v>1339</v>
       </c>
       <c r="V10" s="58" t="n">
         <v>1250</v>
@@ -2950,7 +2950,7 @@
         </is>
       </c>
       <c r="U11" s="58" t="n">
-        <v>1178.32</v>
+        <v>1339</v>
       </c>
       <c r="V11" s="58" t="n">
         <v>1178.32</v>
@@ -3011,7 +3011,7 @@
         </is>
       </c>
       <c r="U12" s="58" t="n">
-        <v>1077.16</v>
+        <v>1339</v>
       </c>
       <c r="V12" s="58" t="n">
         <v>1077.16</v>
@@ -3072,7 +3072,7 @@
         </is>
       </c>
       <c r="U13" s="58" t="n">
-        <v>1071.2</v>
+        <v>1339</v>
       </c>
       <c r="V13" s="58" t="n">
         <v>1071.2</v>
@@ -3133,7 +3133,7 @@
         </is>
       </c>
       <c r="U14" s="58" t="n">
-        <v>1200</v>
+        <v>1339</v>
       </c>
       <c r="V14" s="58" t="n">
         <v>1200</v>
@@ -3194,7 +3194,7 @@
         </is>
       </c>
       <c r="U15" s="58" t="n">
-        <v>964.08</v>
+        <v>1339</v>
       </c>
       <c r="V15" s="58" t="n">
         <v>964.08</v>
@@ -3255,7 +3255,7 @@
         </is>
       </c>
       <c r="U16" s="58" t="n">
-        <v>1200</v>
+        <v>1339</v>
       </c>
       <c r="V16" s="58" t="n">
         <v>1200</v>
@@ -3377,7 +3377,7 @@
         </is>
       </c>
       <c r="U18" s="58" t="n">
-        <v>1200</v>
+        <v>1339</v>
       </c>
       <c r="V18" s="58" t="n">
         <v>1200</v>
@@ -3438,7 +3438,7 @@
         </is>
       </c>
       <c r="U19" s="58" t="n">
-        <v>1200</v>
+        <v>1339</v>
       </c>
       <c r="V19" s="58" t="n">
         <v>1200</v>
@@ -3499,7 +3499,7 @@
         </is>
       </c>
       <c r="U20" s="58" t="n">
-        <v>1300</v>
+        <v>1339</v>
       </c>
       <c r="V20" s="58" t="n">
         <v>1300</v>
@@ -3560,7 +3560,7 @@
         </is>
       </c>
       <c r="U21" s="58" t="n">
-        <v>1250</v>
+        <v>1339</v>
       </c>
       <c r="V21" s="58" t="n">
         <v>1250</v>
@@ -3621,7 +3621,7 @@
         </is>
       </c>
       <c r="U22" s="58" t="n">
-        <v>834.64</v>
+        <v>1339</v>
       </c>
       <c r="V22" s="58" t="n">
         <v>834.64</v>
@@ -3740,7 +3740,7 @@
         </is>
       </c>
       <c r="U24" s="58" t="n">
-        <v>997.8200000000001</v>
+        <v>1339</v>
       </c>
       <c r="V24" s="58" t="n">
         <v>997.8200000000001</v>
@@ -3801,7 +3801,7 @@
         </is>
       </c>
       <c r="U25" s="58" t="n">
-        <v>1040</v>
+        <v>1339</v>
       </c>
       <c r="V25" s="58" t="n">
         <v>1040</v>
@@ -3862,7 +3862,7 @@
         </is>
       </c>
       <c r="U26" s="58" t="n">
-        <v>1250</v>
+        <v>1520</v>
       </c>
       <c r="V26" s="58" t="n">
         <v>0</v>
@@ -3914,7 +3914,7 @@
         </is>
       </c>
       <c r="U27" s="58" t="n">
-        <v>1166.65</v>
+        <v>1520</v>
       </c>
       <c r="V27" s="58" t="n">
         <v>1166.65</v>
@@ -3975,7 +3975,7 @@
         </is>
       </c>
       <c r="U28" s="58" t="n">
-        <v>1200</v>
+        <v>1520</v>
       </c>
       <c r="V28" s="58" t="n">
         <v>1200</v>
@@ -4097,7 +4097,7 @@
         </is>
       </c>
       <c r="U30" s="58" t="n">
-        <v>1250</v>
+        <v>1520</v>
       </c>
       <c r="V30" s="58" t="n">
         <v>1250</v>
@@ -4158,7 +4158,7 @@
         </is>
       </c>
       <c r="U31" s="58" t="n">
-        <v>1210.69</v>
+        <v>1520</v>
       </c>
       <c r="V31" s="58" t="n">
         <v>1210.69</v>
@@ -4219,7 +4219,7 @@
         </is>
       </c>
       <c r="U32" s="58" t="n">
-        <v>1133</v>
+        <v>1520</v>
       </c>
       <c r="V32" s="58" t="n">
         <v>1133</v>
@@ -4280,7 +4280,7 @@
         </is>
       </c>
       <c r="U33" s="58" t="n">
-        <v>1393</v>
+        <v>1520</v>
       </c>
       <c r="V33" s="58" t="n">
         <v>1393</v>
@@ -4341,7 +4341,7 @@
         </is>
       </c>
       <c r="U34" s="58" t="n">
-        <v>1185</v>
+        <v>1520</v>
       </c>
       <c r="V34" s="58" t="n">
         <v>1185</v>
@@ -4402,7 +4402,7 @@
         </is>
       </c>
       <c r="U35" s="58" t="n">
-        <v>1339</v>
+        <v>1520</v>
       </c>
       <c r="V35" s="58" t="n">
         <v>1339</v>
@@ -4463,7 +4463,7 @@
         </is>
       </c>
       <c r="U36" s="58" t="n">
-        <v>1030</v>
+        <v>1520</v>
       </c>
       <c r="V36" s="58" t="n">
         <v>1030</v>
@@ -4524,7 +4524,7 @@
         </is>
       </c>
       <c r="U37" s="58" t="n">
-        <v>1500</v>
+        <v>1520</v>
       </c>
       <c r="V37" s="58" t="n">
         <v>1500</v>
@@ -4585,7 +4585,7 @@
         </is>
       </c>
       <c r="U38" s="58" t="n">
-        <v>1300</v>
+        <v>1520</v>
       </c>
       <c r="V38" s="58" t="n">
         <v>1300</v>
@@ -4646,7 +4646,7 @@
         </is>
       </c>
       <c r="U39" s="58" t="n">
-        <v>888.64</v>
+        <v>1520</v>
       </c>
       <c r="V39" s="58" t="n">
         <v>888.64</v>
@@ -4707,7 +4707,7 @@
         </is>
       </c>
       <c r="U40" s="58" t="n">
-        <v>1250</v>
+        <v>1520</v>
       </c>
       <c r="V40" s="58" t="n">
         <v>1250</v>
@@ -4768,7 +4768,7 @@
         </is>
       </c>
       <c r="U41" s="58" t="n">
-        <v>1236</v>
+        <v>1520</v>
       </c>
       <c r="V41" s="58" t="n">
         <v>1236</v>
@@ -4829,7 +4829,7 @@
         </is>
       </c>
       <c r="U42" s="58" t="n">
-        <v>1442</v>
+        <v>1520</v>
       </c>
       <c r="V42" s="58" t="n">
         <v>1442</v>
@@ -4890,7 +4890,7 @@
         </is>
       </c>
       <c r="U43" s="58" t="n">
-        <v>1200</v>
+        <v>1520</v>
       </c>
       <c r="V43" s="58" t="n">
         <v>1200</v>
@@ -4951,7 +4951,7 @@
         </is>
       </c>
       <c r="U44" s="58" t="n">
-        <v>1400</v>
+        <v>1520</v>
       </c>
       <c r="V44" s="58" t="n">
         <v>1400</v>
@@ -5012,7 +5012,7 @@
         </is>
       </c>
       <c r="U45" s="58" t="n">
-        <v>1232</v>
+        <v>1520</v>
       </c>
       <c r="V45" s="58" t="n">
         <v>1232</v>
@@ -5073,7 +5073,7 @@
         </is>
       </c>
       <c r="U46" s="58" t="n">
-        <v>751.87</v>
+        <v>1520</v>
       </c>
       <c r="V46" s="58" t="n">
         <v>751.87</v>
@@ -5134,7 +5134,7 @@
         </is>
       </c>
       <c r="U47" s="58" t="n">
-        <v>1250</v>
+        <v>1520</v>
       </c>
       <c r="V47" s="58" t="n">
         <v>1250</v>
@@ -5195,7 +5195,7 @@
         </is>
       </c>
       <c r="U48" s="58" t="n">
-        <v>1150</v>
+        <v>1520</v>
       </c>
       <c r="V48" s="58" t="n">
         <v>1150</v>
@@ -5256,7 +5256,7 @@
         </is>
       </c>
       <c r="U49" s="58" t="n">
-        <v>1442</v>
+        <v>1849</v>
       </c>
       <c r="V49" s="58" t="n">
         <v>1442</v>
@@ -5317,7 +5317,7 @@
         </is>
       </c>
       <c r="U50" s="58" t="n">
-        <v>1327</v>
+        <v>1849</v>
       </c>
       <c r="V50" s="58" t="n">
         <v>1327</v>
@@ -5378,7 +5378,7 @@
         </is>
       </c>
       <c r="U51" s="58" t="n">
-        <v>1300</v>
+        <v>1849</v>
       </c>
       <c r="V51" s="58" t="n">
         <v>1300</v>
@@ -5439,7 +5439,7 @@
         </is>
       </c>
       <c r="U52" s="58" t="n">
-        <v>1674</v>
+        <v>1849</v>
       </c>
       <c r="V52" s="58" t="n">
         <v>1674</v>
@@ -5500,7 +5500,7 @@
         </is>
       </c>
       <c r="U53" s="58" t="n">
-        <v>1200</v>
+        <v>1849</v>
       </c>
       <c r="V53" s="58" t="n">
         <v>1200</v>
@@ -5622,7 +5622,7 @@
         </is>
       </c>
       <c r="U55" s="58" t="n">
-        <v>1236</v>
+        <v>1849</v>
       </c>
       <c r="V55" s="58" t="n">
         <v>1236</v>
@@ -5683,7 +5683,7 @@
         </is>
       </c>
       <c r="U56" s="58" t="n">
-        <v>1339.9</v>
+        <v>1849</v>
       </c>
       <c r="V56" s="58" t="n">
         <v>1339.9</v>
@@ -5744,7 +5744,7 @@
         </is>
       </c>
       <c r="U57" s="58" t="n">
-        <v>1700</v>
+        <v>1849</v>
       </c>
       <c r="V57" s="58" t="n">
         <v>1700</v>
@@ -5805,7 +5805,7 @@
         </is>
       </c>
       <c r="U58" s="58" t="n">
-        <v>1236</v>
+        <v>1849</v>
       </c>
       <c r="V58" s="58" t="n">
         <v>1236</v>
@@ -5866,7 +5866,7 @@
         </is>
       </c>
       <c r="U59" s="58" t="n">
-        <v>1500</v>
+        <v>1849</v>
       </c>
       <c r="V59" s="58" t="n">
         <v>1500</v>
@@ -5927,7 +5927,7 @@
         </is>
       </c>
       <c r="U60" s="58" t="n">
-        <v>1650</v>
+        <v>1849</v>
       </c>
       <c r="V60" s="58" t="n">
         <v>1650</v>
@@ -5988,7 +5988,7 @@
         </is>
       </c>
       <c r="U61" s="58" t="n">
-        <v>1400</v>
+        <v>1463.42</v>
       </c>
       <c r="V61" s="58" t="n">
         <v>0</v>
@@ -6040,7 +6040,7 @@
         </is>
       </c>
       <c r="U62" s="58" t="n">
-        <v>1350</v>
+        <v>1463.42</v>
       </c>
       <c r="V62" s="58" t="n">
         <v>1350</v>
@@ -6101,7 +6101,7 @@
         </is>
       </c>
       <c r="U63" s="58" t="n">
-        <v>889.1</v>
+        <v>1463.42</v>
       </c>
       <c r="V63" s="58" t="n">
         <v>889.1</v>
@@ -6162,7 +6162,7 @@
         </is>
       </c>
       <c r="U64" s="58" t="n">
-        <v>1037.83</v>
+        <v>1463.42</v>
       </c>
       <c r="V64" s="58" t="n">
         <v>1037.83</v>
@@ -6284,7 +6284,7 @@
         </is>
       </c>
       <c r="U66" s="58" t="n">
-        <v>1006.21</v>
+        <v>1463.42</v>
       </c>
       <c r="V66" s="58" t="n">
         <v>1006.21</v>
@@ -6345,7 +6345,7 @@
         </is>
       </c>
       <c r="U67" s="58" t="n">
-        <v>1300</v>
+        <v>1463.42</v>
       </c>
       <c r="V67" s="58" t="n">
         <v>1300</v>
@@ -6406,7 +6406,7 @@
         </is>
       </c>
       <c r="U68" s="58" t="n">
-        <v>1302</v>
+        <v>1463.42</v>
       </c>
       <c r="V68" s="58" t="n">
         <v>1302</v>
@@ -6467,7 +6467,7 @@
         </is>
       </c>
       <c r="U69" s="58" t="n">
-        <v>1301</v>
+        <v>1463.42</v>
       </c>
       <c r="V69" s="58" t="n">
         <v>1301</v>
@@ -6528,7 +6528,7 @@
         </is>
       </c>
       <c r="U70" s="58" t="n">
-        <v>1100</v>
+        <v>1463.42</v>
       </c>
       <c r="V70" s="58" t="n">
         <v>1100</v>
@@ -6589,7 +6589,7 @@
         </is>
       </c>
       <c r="U71" s="58" t="n">
-        <v>1400</v>
+        <v>1463.42</v>
       </c>
       <c r="V71" s="58" t="n">
         <v>1400</v>
@@ -6650,7 +6650,7 @@
         </is>
       </c>
       <c r="U72" s="58" t="n">
-        <v>300</v>
+        <v>1463.42</v>
       </c>
       <c r="V72" s="58" t="n">
         <v>300</v>
@@ -6711,7 +6711,7 @@
         </is>
       </c>
       <c r="U73" s="58" t="n">
-        <v>1037.83</v>
+        <v>1463.42</v>
       </c>
       <c r="V73" s="58" t="n">
         <v>1037.83</v>
@@ -6772,7 +6772,7 @@
         </is>
       </c>
       <c r="U74" s="58" t="n">
-        <v>911.76</v>
+        <v>1463.42</v>
       </c>
       <c r="V74" s="58" t="n">
         <v>911.76</v>
@@ -6833,7 +6833,7 @@
         </is>
       </c>
       <c r="U75" s="58" t="n">
-        <v>1350</v>
+        <v>1463.42</v>
       </c>
       <c r="V75" s="58" t="n">
         <v>1350</v>
@@ -6894,7 +6894,7 @@
         </is>
       </c>
       <c r="U76" s="58" t="n">
-        <v>1097.67</v>
+        <v>1463.42</v>
       </c>
       <c r="V76" s="58" t="n">
         <v>1097.67</v>
@@ -6955,7 +6955,7 @@
         </is>
       </c>
       <c r="U77" s="58" t="n">
-        <v>1358</v>
+        <v>1463.42</v>
       </c>
       <c r="V77" s="58" t="n">
         <v>1358</v>
@@ -7016,7 +7016,7 @@
         </is>
       </c>
       <c r="U78" s="58" t="n">
-        <v>1180.69</v>
+        <v>1463.42</v>
       </c>
       <c r="V78" s="58" t="n">
         <v>1180.69</v>
@@ -7077,7 +7077,7 @@
         </is>
       </c>
       <c r="U79" s="58" t="n">
-        <v>1037.83</v>
+        <v>1463.42</v>
       </c>
       <c r="V79" s="58" t="n">
         <v>1037.83</v>
@@ -7138,7 +7138,7 @@
         </is>
       </c>
       <c r="U80" s="58" t="n">
-        <v>806.49</v>
+        <v>1463.42</v>
       </c>
       <c r="V80" s="58" t="n">
         <v>806.49</v>
@@ -7190,7 +7190,7 @@
       <c r="S81" s="61" t="n"/>
       <c r="T81" s="61" t="n"/>
       <c r="U81" s="64" t="n">
-        <v>89302.80000000002</v>
+        <v>110518.4</v>
       </c>
       <c r="V81" s="64" t="n">
         <v>84152.8</v>
@@ -7903,7 +7903,7 @@
         </is>
       </c>
       <c r="L32" s="82" t="n">
-        <v>1250</v>
+        <v>1339</v>
       </c>
       <c r="M32" s="82">
         <f>Y32</f>
@@ -7978,7 +7978,7 @@
         </is>
       </c>
       <c r="L33" s="82" t="n">
-        <v>1250</v>
+        <v>1339</v>
       </c>
       <c r="M33" s="82">
         <f>Y33</f>
@@ -8053,7 +8053,7 @@
         </is>
       </c>
       <c r="L34" s="85" t="n">
-        <v>1250</v>
+        <v>1339</v>
       </c>
       <c r="M34" s="85">
         <f>Y34</f>
@@ -8129,7 +8129,7 @@
         </is>
       </c>
       <c r="L35" s="85" t="n">
-        <v>1178.32</v>
+        <v>1339</v>
       </c>
       <c r="M35" s="85">
         <f>Y35</f>
@@ -8205,7 +8205,7 @@
         </is>
       </c>
       <c r="L36" s="85" t="n">
-        <v>1077.16</v>
+        <v>1339</v>
       </c>
       <c r="M36" s="85">
         <f>Y36</f>
@@ -8281,7 +8281,7 @@
         </is>
       </c>
       <c r="L37" s="85" t="n">
-        <v>1071.2</v>
+        <v>1339</v>
       </c>
       <c r="M37" s="85">
         <f>Y37</f>
@@ -8357,7 +8357,7 @@
         </is>
       </c>
       <c r="L38" s="85" t="n">
-        <v>1200</v>
+        <v>1339</v>
       </c>
       <c r="M38" s="85">
         <f>Y38</f>
@@ -8433,7 +8433,7 @@
         </is>
       </c>
       <c r="L39" s="85" t="n">
-        <v>964.08</v>
+        <v>1339</v>
       </c>
       <c r="M39" s="85">
         <f>Y39</f>
@@ -8509,7 +8509,7 @@
         </is>
       </c>
       <c r="L40" s="85" t="n">
-        <v>1200</v>
+        <v>1339</v>
       </c>
       <c r="M40" s="85">
         <f>Y40</f>
@@ -8661,7 +8661,7 @@
         </is>
       </c>
       <c r="L42" s="85" t="n">
-        <v>1200</v>
+        <v>1339</v>
       </c>
       <c r="M42" s="85">
         <f>Y42</f>
@@ -8737,7 +8737,7 @@
         </is>
       </c>
       <c r="L43" s="85" t="n">
-        <v>1200</v>
+        <v>1339</v>
       </c>
       <c r="M43" s="85">
         <f>Y43</f>
@@ -8813,7 +8813,7 @@
         </is>
       </c>
       <c r="L44" s="85" t="n">
-        <v>1300</v>
+        <v>1339</v>
       </c>
       <c r="M44" s="85">
         <f>Y44</f>
@@ -8889,7 +8889,7 @@
         </is>
       </c>
       <c r="L45" s="85" t="n">
-        <v>1250</v>
+        <v>1339</v>
       </c>
       <c r="M45" s="85">
         <f>Y45</f>
@@ -8965,7 +8965,7 @@
         </is>
       </c>
       <c r="L46" s="85" t="n">
-        <v>834.64</v>
+        <v>1339</v>
       </c>
       <c r="M46" s="85">
         <f>Y46</f>
@@ -9114,7 +9114,7 @@
         </is>
       </c>
       <c r="L48" s="85" t="n">
-        <v>997.8200000000001</v>
+        <v>1339</v>
       </c>
       <c r="M48" s="85">
         <f>Y48</f>
@@ -9190,7 +9190,7 @@
         </is>
       </c>
       <c r="L49" s="85" t="n">
-        <v>1040</v>
+        <v>1339</v>
       </c>
       <c r="M49" s="85">
         <f>Y49</f>
@@ -9266,7 +9266,7 @@
         </is>
       </c>
       <c r="L50" s="82" t="n">
-        <v>1250</v>
+        <v>1520</v>
       </c>
       <c r="M50" s="82">
         <f>Y50</f>
@@ -9341,7 +9341,7 @@
         </is>
       </c>
       <c r="L51" s="85" t="n">
-        <v>1166.65</v>
+        <v>1520</v>
       </c>
       <c r="M51" s="85">
         <f>Y51</f>
@@ -9417,7 +9417,7 @@
         </is>
       </c>
       <c r="L52" s="85" t="n">
-        <v>1200</v>
+        <v>1520</v>
       </c>
       <c r="M52" s="85">
         <f>Y52</f>
@@ -9569,7 +9569,7 @@
         </is>
       </c>
       <c r="L54" s="85" t="n">
-        <v>1250</v>
+        <v>1520</v>
       </c>
       <c r="M54" s="85">
         <f>Y54</f>
@@ -9645,7 +9645,7 @@
         </is>
       </c>
       <c r="L55" s="85" t="n">
-        <v>1210.69</v>
+        <v>1520</v>
       </c>
       <c r="M55" s="85">
         <f>Y55</f>
@@ -9721,7 +9721,7 @@
         </is>
       </c>
       <c r="L56" s="85" t="n">
-        <v>1133</v>
+        <v>1520</v>
       </c>
       <c r="M56" s="85">
         <f>Y56</f>
@@ -9797,7 +9797,7 @@
         </is>
       </c>
       <c r="L57" s="85" t="n">
-        <v>1393</v>
+        <v>1520</v>
       </c>
       <c r="M57" s="85">
         <f>Y57</f>
@@ -9873,7 +9873,7 @@
         </is>
       </c>
       <c r="L58" s="85" t="n">
-        <v>1185</v>
+        <v>1520</v>
       </c>
       <c r="M58" s="85">
         <f>Y58</f>
@@ -9949,7 +9949,7 @@
         </is>
       </c>
       <c r="L59" s="85" t="n">
-        <v>1339</v>
+        <v>1520</v>
       </c>
       <c r="M59" s="85">
         <f>Y59</f>
@@ -10025,7 +10025,7 @@
         </is>
       </c>
       <c r="L60" s="85" t="n">
-        <v>1030</v>
+        <v>1520</v>
       </c>
       <c r="M60" s="85">
         <f>Y60</f>
@@ -10101,7 +10101,7 @@
         </is>
       </c>
       <c r="L61" s="85" t="n">
-        <v>1500</v>
+        <v>1520</v>
       </c>
       <c r="M61" s="85">
         <f>Y61</f>
@@ -10177,7 +10177,7 @@
         </is>
       </c>
       <c r="L62" s="85" t="n">
-        <v>1300</v>
+        <v>1520</v>
       </c>
       <c r="M62" s="85">
         <f>Y62</f>
@@ -10253,7 +10253,7 @@
         </is>
       </c>
       <c r="L63" s="85" t="n">
-        <v>888.64</v>
+        <v>1520</v>
       </c>
       <c r="M63" s="85">
         <f>Y63</f>
@@ -10329,7 +10329,7 @@
         </is>
       </c>
       <c r="L64" s="85" t="n">
-        <v>1250</v>
+        <v>1520</v>
       </c>
       <c r="M64" s="85">
         <f>Y64</f>
@@ -10405,7 +10405,7 @@
         </is>
       </c>
       <c r="L65" s="85" t="n">
-        <v>1236</v>
+        <v>1520</v>
       </c>
       <c r="M65" s="85">
         <f>Y65</f>
@@ -10481,7 +10481,7 @@
         </is>
       </c>
       <c r="L66" s="85" t="n">
-        <v>1442</v>
+        <v>1520</v>
       </c>
       <c r="M66" s="85">
         <f>Y66</f>
@@ -10557,7 +10557,7 @@
         </is>
       </c>
       <c r="L67" s="85" t="n">
-        <v>1200</v>
+        <v>1520</v>
       </c>
       <c r="M67" s="85">
         <f>Y67</f>
@@ -10633,7 +10633,7 @@
         </is>
       </c>
       <c r="L68" s="85" t="n">
-        <v>1400</v>
+        <v>1520</v>
       </c>
       <c r="M68" s="85">
         <f>Y68</f>
@@ -10709,7 +10709,7 @@
         </is>
       </c>
       <c r="L69" s="85" t="n">
-        <v>1232</v>
+        <v>1520</v>
       </c>
       <c r="M69" s="85">
         <f>Y69</f>
@@ -10785,7 +10785,7 @@
         </is>
       </c>
       <c r="L70" s="85" t="n">
-        <v>751.87</v>
+        <v>1520</v>
       </c>
       <c r="M70" s="85">
         <f>Y70</f>
@@ -10861,7 +10861,7 @@
         </is>
       </c>
       <c r="L71" s="85" t="n">
-        <v>1250</v>
+        <v>1520</v>
       </c>
       <c r="M71" s="85">
         <f>Y71</f>
@@ -10937,7 +10937,7 @@
         </is>
       </c>
       <c r="L72" s="85" t="n">
-        <v>1150</v>
+        <v>1520</v>
       </c>
       <c r="M72" s="85">
         <f>Y72</f>
@@ -11013,7 +11013,7 @@
         </is>
       </c>
       <c r="L73" s="85" t="n">
-        <v>1442</v>
+        <v>1849</v>
       </c>
       <c r="M73" s="85">
         <f>Y73</f>
@@ -11089,7 +11089,7 @@
         </is>
       </c>
       <c r="L74" s="85" t="n">
-        <v>1327</v>
+        <v>1849</v>
       </c>
       <c r="M74" s="85">
         <f>Y74</f>
@@ -11165,7 +11165,7 @@
         </is>
       </c>
       <c r="L75" s="85" t="n">
-        <v>1300</v>
+        <v>1849</v>
       </c>
       <c r="M75" s="85">
         <f>Y75</f>
@@ -11241,7 +11241,7 @@
         </is>
       </c>
       <c r="L76" s="85" t="n">
-        <v>1674</v>
+        <v>1849</v>
       </c>
       <c r="M76" s="85">
         <f>Y76</f>
@@ -11317,7 +11317,7 @@
         </is>
       </c>
       <c r="L77" s="85" t="n">
-        <v>1200</v>
+        <v>1849</v>
       </c>
       <c r="M77" s="85">
         <f>Y77</f>
@@ -11469,7 +11469,7 @@
         </is>
       </c>
       <c r="L79" s="85" t="n">
-        <v>1236</v>
+        <v>1849</v>
       </c>
       <c r="M79" s="85">
         <f>Y79</f>
@@ -11545,7 +11545,7 @@
         </is>
       </c>
       <c r="L80" s="85" t="n">
-        <v>1339.9</v>
+        <v>1849</v>
       </c>
       <c r="M80" s="85">
         <f>Y80</f>
@@ -11621,7 +11621,7 @@
         </is>
       </c>
       <c r="L81" s="85" t="n">
-        <v>1700</v>
+        <v>1849</v>
       </c>
       <c r="M81" s="85">
         <f>Y81</f>
@@ -11697,7 +11697,7 @@
         </is>
       </c>
       <c r="L82" s="85" t="n">
-        <v>1236</v>
+        <v>1849</v>
       </c>
       <c r="M82" s="85">
         <f>Y82</f>
@@ -11773,7 +11773,7 @@
         </is>
       </c>
       <c r="L83" s="85" t="n">
-        <v>1500</v>
+        <v>1849</v>
       </c>
       <c r="M83" s="85">
         <f>Y83</f>
@@ -11849,7 +11849,7 @@
         </is>
       </c>
       <c r="L84" s="85" t="n">
-        <v>1650</v>
+        <v>1849</v>
       </c>
       <c r="M84" s="85">
         <f>Y84</f>
@@ -11925,7 +11925,7 @@
         </is>
       </c>
       <c r="L85" s="82" t="n">
-        <v>1400</v>
+        <v>1463.42</v>
       </c>
       <c r="M85" s="82">
         <f>Y85</f>
@@ -12000,7 +12000,7 @@
         </is>
       </c>
       <c r="L86" s="85" t="n">
-        <v>1350</v>
+        <v>1463.42</v>
       </c>
       <c r="M86" s="85">
         <f>Y86</f>
@@ -12076,7 +12076,7 @@
         </is>
       </c>
       <c r="L87" s="85" t="n">
-        <v>889.1</v>
+        <v>1463.42</v>
       </c>
       <c r="M87" s="85">
         <f>Y87</f>
@@ -12152,7 +12152,7 @@
         </is>
       </c>
       <c r="L88" s="85" t="n">
-        <v>1037.83</v>
+        <v>1463.42</v>
       </c>
       <c r="M88" s="85">
         <f>Y88</f>
@@ -12304,7 +12304,7 @@
         </is>
       </c>
       <c r="L90" s="85" t="n">
-        <v>1006.21</v>
+        <v>1463.42</v>
       </c>
       <c r="M90" s="85">
         <f>Y90</f>
@@ -12380,7 +12380,7 @@
         </is>
       </c>
       <c r="L91" s="85" t="n">
-        <v>1300</v>
+        <v>1463.42</v>
       </c>
       <c r="M91" s="85">
         <f>Y91</f>
@@ -12456,7 +12456,7 @@
         </is>
       </c>
       <c r="L92" s="85" t="n">
-        <v>1302</v>
+        <v>1463.42</v>
       </c>
       <c r="M92" s="85">
         <f>Y92</f>
@@ -12532,7 +12532,7 @@
         </is>
       </c>
       <c r="L93" s="85" t="n">
-        <v>1301</v>
+        <v>1463.42</v>
       </c>
       <c r="M93" s="85">
         <f>Y93</f>
@@ -12608,7 +12608,7 @@
         </is>
       </c>
       <c r="L94" s="85" t="n">
-        <v>1100</v>
+        <v>1463.42</v>
       </c>
       <c r="M94" s="85">
         <f>Y94</f>
@@ -12684,7 +12684,7 @@
         </is>
       </c>
       <c r="L95" s="85" t="n">
-        <v>1400</v>
+        <v>1463.42</v>
       </c>
       <c r="M95" s="85">
         <f>Y95</f>
@@ -12760,7 +12760,7 @@
         </is>
       </c>
       <c r="L96" s="85" t="n">
-        <v>300</v>
+        <v>1463.42</v>
       </c>
       <c r="M96" s="85">
         <f>Y96</f>
@@ -12836,7 +12836,7 @@
         </is>
       </c>
       <c r="L97" s="85" t="n">
-        <v>1037.83</v>
+        <v>1463.42</v>
       </c>
       <c r="M97" s="85">
         <f>Y97</f>
@@ -12912,7 +12912,7 @@
         </is>
       </c>
       <c r="L98" s="85" t="n">
-        <v>911.76</v>
+        <v>1463.42</v>
       </c>
       <c r="M98" s="85">
         <f>Y98</f>
@@ -12988,7 +12988,7 @@
         </is>
       </c>
       <c r="L99" s="85" t="n">
-        <v>1350</v>
+        <v>1463.42</v>
       </c>
       <c r="M99" s="85">
         <f>Y99</f>
@@ -13064,7 +13064,7 @@
         </is>
       </c>
       <c r="L100" s="85" t="n">
-        <v>1097.67</v>
+        <v>1463.42</v>
       </c>
       <c r="M100" s="85">
         <f>Y100</f>
@@ -13140,7 +13140,7 @@
         </is>
       </c>
       <c r="L101" s="85" t="n">
-        <v>1358</v>
+        <v>1463.42</v>
       </c>
       <c r="M101" s="85">
         <f>Y101</f>
@@ -13216,7 +13216,7 @@
         </is>
       </c>
       <c r="L102" s="85" t="n">
-        <v>1180.69</v>
+        <v>1463.42</v>
       </c>
       <c r="M102" s="85">
         <f>Y102</f>
@@ -13292,7 +13292,7 @@
         </is>
       </c>
       <c r="L103" s="85" t="n">
-        <v>1037.83</v>
+        <v>1463.42</v>
       </c>
       <c r="M103" s="85">
         <f>Y103</f>
@@ -13368,7 +13368,7 @@
         </is>
       </c>
       <c r="L104" s="85" t="n">
-        <v>806.49</v>
+        <v>1463.42</v>
       </c>
       <c r="M104" s="85">
         <f>Y104</f>

</xml_diff>